<commit_message>
Revert "new questions in xlsx"
This reverts commit 1513d2bc0d54b260a5ccdb7da970a5986692d25d.
</commit_message>
<xml_diff>
--- a/experiment_implementation/data/participant_questionnaire_toy_x_1/multipleye_questionnaire_questions_toy.xlsx
+++ b/experiment_implementation/data/participant_questionnaire_toy_x_1/multipleye_questionnaire_questions_toy.xlsx
@@ -1,29 +1,49 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maros/Documents/wg1-experiment-implementation/experiment_implementation/data/participant_questionnaire_toy_x_1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/debor/repos/wg1-experiment-implementation/experiment_implementation/data/participant_questionnaire_toy_x_1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70D367F8-0E5D-9743-913C-C39325AFC8F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4D22396-22AA-CC41-BBE8-45448568E13B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="29920" windowHeight="18660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="multipleye_questionnaire_questi" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">multipleye_questionnaire_questi!$A$1:$P$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">multipleye_questionnaire_questi!$A$1:$P$27</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={D353FB44-2422-FEF8-3AB3-E3F2443958F3}</author>
+  </authors>
+  <commentList>
+    <comment ref="B3" authorId="0" shapeId="0" xr:uid="{D353FB44-2422-FEF8-3AB3-E3F2443958F3}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    than [insert current language]?
+Reply:
+    Hi, everyone who is going to translate this column, we don't need to specify any languages here. It is enough to say "do you read in any other language(s)?" A menu with language options is not needed because it will read the language options from the iso file directly. (Cui)</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="130">
   <si>
     <t>pq_question_no</t>
   </si>
@@ -94,9 +114,27 @@
     <t>dropdown</t>
   </si>
   <si>
+    <t>Years of education</t>
+  </si>
+  <si>
+    <t>1;20</t>
+  </si>
+  <si>
+    <t>&gt;20 years</t>
+  </si>
+  <si>
+    <t>Please consider the years of education starting with primary school (excluding pre-school and kindergarten), including PhD studies.</t>
+  </si>
+  <si>
+    <t>years_education</t>
+  </si>
+  <si>
     <t>interval</t>
   </si>
   <si>
+    <t>2a</t>
+  </si>
+  <si>
     <t>Please report the highest level of education you have completed</t>
   </si>
   <si>
@@ -133,9 +171,30 @@
     <t>Age</t>
   </si>
   <si>
+    <t>18;120</t>
+  </si>
+  <si>
+    <t>Please provide you age (in number of years). The allowed values are from 18 to 120.</t>
+  </si>
+  <si>
     <t>age</t>
   </si>
   <si>
+    <t>Compared to the other people in your geographical community, how do you rate your socio-economic status?</t>
+  </si>
+  <si>
+    <t>below-average</t>
+  </si>
+  <si>
+    <t>average</t>
+  </si>
+  <si>
+    <t>above-average</t>
+  </si>
+  <si>
+    <t>socio_economic_status</t>
+  </si>
+  <si>
     <t>As a child, did you grow up with one or multiple languages at the same time?</t>
   </si>
   <si>
@@ -154,15 +213,30 @@
     <t>childhood_languages</t>
   </si>
   <si>
+    <t>Native language: What is the first language you learned as a child?</t>
+  </si>
+  <si>
     <t>native_language_1</t>
   </si>
   <si>
     <t>dropdown_file</t>
   </si>
   <si>
+    <t>Which other language(s) did you grow up with?</t>
+  </si>
+  <si>
+    <t>native_language</t>
+  </si>
+  <si>
+    <t>Language of use: Which language do you currently use the most?</t>
+  </si>
+  <si>
     <t>use_language</t>
   </si>
   <si>
+    <t>Dominant language: Which language are you currently the most at ease with?</t>
+  </si>
+  <si>
     <t>dominant_language</t>
   </si>
   <si>
@@ -181,6 +255,12 @@
     <t>read_language</t>
   </si>
   <si>
+    <t>11a</t>
+  </si>
+  <si>
+    <t>Academic materials</t>
+  </si>
+  <si>
     <t>0 hours</t>
   </si>
   <si>
@@ -196,21 +276,66 @@
     <t>More than 5 hours</t>
   </si>
   <si>
+    <t>academic_reading_time</t>
+  </si>
+  <si>
+    <t>11b</t>
+  </si>
+  <si>
+    <t>Magazines</t>
+  </si>
+  <si>
+    <t>magazine_reading_time</t>
+  </si>
+  <si>
+    <t>11c</t>
+  </si>
+  <si>
+    <t>Newspapers</t>
+  </si>
+  <si>
     <t>newspaper_reading_time</t>
   </si>
   <si>
+    <t>11d</t>
+  </si>
+  <si>
+    <t>E-mails</t>
+  </si>
+  <si>
+    <t>email_reading_time</t>
+  </si>
+  <si>
+    <t>11e</t>
+  </si>
+  <si>
     <t>Fiction books</t>
   </si>
   <si>
     <t>fiction_reading_time</t>
   </si>
   <si>
+    <t>11f</t>
+  </si>
+  <si>
     <t>Nonfiction/ special interest books</t>
   </si>
   <si>
     <t>nonfiction_reading_time</t>
   </si>
   <si>
+    <t>11g</t>
+  </si>
+  <si>
+    <t>Internet media (including social media, forums, and blogs)</t>
+  </si>
+  <si>
+    <t>internet_reading_time</t>
+  </si>
+  <si>
+    <t>11h</t>
+  </si>
+  <si>
     <t>Other categories</t>
   </si>
   <si>
@@ -295,6 +420,9 @@
     <t>alcohol_today</t>
   </si>
   <si>
+    <t>10a</t>
+  </si>
+  <si>
     <t>Please specify the dialects:</t>
   </si>
   <si>
@@ -305,112 +433,13 @@
   </si>
   <si>
     <t>Do you read in any other language(s)?</t>
-  </si>
-  <si>
-    <t>Newspapers and magazines</t>
-  </si>
-  <si>
-    <t>Online content (e-mails, social media, forums, …)</t>
-  </si>
-  <si>
-    <t>Which languages did you use in your middle age?</t>
-  </si>
-  <si>
-    <t>What is the first language you learned as a child?</t>
-  </si>
-  <si>
-    <t>Which language do you currently use the most?</t>
-  </si>
-  <si>
-    <t>Which language are you currently the most at ease with?</t>
-  </si>
-  <si>
-    <t>education_language</t>
-  </si>
-  <si>
-    <t>middle_age_language</t>
-  </si>
-  <si>
-    <t>online_reading_time</t>
-  </si>
-  <si>
-    <t>Which languages did you use in your educational settings?</t>
-  </si>
-  <si>
-    <t>How many years have you been in retirement?</t>
-  </si>
-  <si>
-    <t>retirement_years</t>
-  </si>
-  <si>
-    <t>0;50</t>
-  </si>
-  <si>
-    <t>impairments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Do you have any medical conditions, particularly neurocognitive or language-related impairments? </t>
-  </si>
-  <si>
-    <t>Which other language(s) did you grow up with?</t>
-  </si>
-  <si>
-    <t>native_language</t>
-  </si>
-  <si>
-    <t>14a</t>
-  </si>
-  <si>
-    <t>30;120</t>
-  </si>
-  <si>
-    <t>Please provide you age (in number of years). The allowed values are from 30 to 120.</t>
-  </si>
-  <si>
-    <t>5a</t>
-  </si>
-  <si>
-    <t>15a</t>
-  </si>
-  <si>
-    <t>15b</t>
-  </si>
-  <si>
-    <t>15c</t>
-  </si>
-  <si>
-    <t>15d</t>
-  </si>
-  <si>
-    <t>15e</t>
-  </si>
-  <si>
-    <t>medication</t>
-  </si>
-  <si>
-    <t>6a</t>
-  </si>
-  <si>
-    <t>Please specify your medical conditions:</t>
-  </si>
-  <si>
-    <t>Please specify the medications:</t>
-  </si>
-  <si>
-    <t>Do you take any medications?</t>
-  </si>
-  <si>
-    <t>impairments_detail</t>
-  </si>
-  <si>
-    <t>medication_detail</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -427,12 +456,6 @@
       <color rgb="FF1D1C1D"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -455,7 +478,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -472,7 +495,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -488,6 +510,13 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Stefan Frank (Gastgebruiker)" id="{F9E47CF5-FABA-A131-AD4D-74C918431CC5}" userId="uid-1704869221436" providerId="Teamlab"/>
+  <person displayName="Cui Ding" id="{A0F657DF-FEB6-C44A-9013-0FF546126BA2}" userId="S::cui.ding@uzh.ch::c3b316e5-323e-462a-8a16-67367b714826" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -718,14 +747,34 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="B3" dT="2024-07-15T15:00:22.01" personId="{F9E47CF5-FABA-A131-AD4D-74C918431CC5}" id="{D353FB44-2422-FEF8-3AB3-E3F2443958F3}">
+    <text xml:space="preserve">than [insert current language]?
+</text>
+  </threadedComment>
+  <threadedComment ref="B3" dT="2024-11-05T15:38:32.36" personId="{A0F657DF-FEB6-C44A-9013-0FF546126BA2}" id="{74697B6F-5D15-6F47-8BD5-5BA580D1B4BE}" parentId="{D353FB44-2422-FEF8-3AB3-E3F2443958F3}">
+    <text>Hi, everyone who is going to translate this column, we don't need to specify any languages here. It is enough to say "do you read in any other language(s)?" A menu with language options is not needed because it will read the language options from the iso file directly. (Cui)</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P33"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:P27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="56.1640625" customWidth="1"/>
-    <col min="3" max="13" width="3.33203125" customWidth="1"/>
-    <col min="14" max="14" width="5.6640625" customWidth="1"/>
+    <col min="2" max="2" width="96.1640625" customWidth="1"/>
+    <col min="3" max="3" width="39.83203125" customWidth="1"/>
+    <col min="4" max="5" width="23.5" customWidth="1"/>
+    <col min="6" max="6" width="24.83203125" customWidth="1"/>
+    <col min="7" max="7" width="32.1640625" customWidth="1"/>
+    <col min="8" max="8" width="25.5" customWidth="1"/>
+    <col min="9" max="9" width="19.83203125" customWidth="1"/>
+    <col min="10" max="10" width="19.1640625" customWidth="1"/>
+    <col min="11" max="11" width="54" customWidth="1"/>
+    <col min="12" max="12" width="35.1640625" customWidth="1"/>
+    <col min="13" max="13" width="31.6640625" customWidth="1"/>
     <col min="15" max="15" width="52.5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -780,135 +829,130 @@
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>1</v>
+      <c r="A2" t="s">
+        <v>70</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>72</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>73</v>
       </c>
       <c r="E2" t="s">
-        <v>19</v>
+        <v>74</v>
       </c>
       <c r="F2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G2" t="s">
+        <v>76</v>
+      </c>
+      <c r="N2">
+        <v>1</v>
+      </c>
+      <c r="O2" t="s">
+        <v>77</v>
+      </c>
+      <c r="P2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A3">
         <v>20</v>
       </c>
-      <c r="N2">
-        <v>1</v>
-      </c>
-      <c r="O2" t="s">
-        <v>21</v>
-      </c>
-      <c r="P2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="L3" s="4"/>
-      <c r="M3" s="1"/>
-      <c r="N3" s="1">
-        <v>1</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="P3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B3" t="s">
+        <v>129</v>
+      </c>
+      <c r="M3" t="s">
+        <v>99</v>
+      </c>
+      <c r="N3">
+        <v>1</v>
+      </c>
+      <c r="O3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="17" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C4" t="s">
-        <v>112</v>
+        <v>42</v>
       </c>
       <c r="M4" t="s">
-        <v>113</v>
+        <v>43</v>
       </c>
       <c r="N4">
         <v>1</v>
       </c>
       <c r="O4" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="P4" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="B5" t="s">
-        <v>104</v>
+        <v>122</v>
       </c>
       <c r="C5" t="s">
-        <v>106</v>
+        <v>123</v>
+      </c>
+      <c r="D5" t="s">
+        <v>118</v>
+      </c>
+      <c r="E5" t="s">
+        <v>119</v>
+      </c>
+      <c r="M5" t="s">
+        <v>120</v>
       </c>
       <c r="N5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O5" t="s">
-        <v>105</v>
+        <v>124</v>
       </c>
       <c r="P5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>108</v>
+        <v>117</v>
+      </c>
+      <c r="C6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E6" t="s">
+        <v>119</v>
+      </c>
+      <c r="M6" t="s">
+        <v>120</v>
       </c>
       <c r="N6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O6" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="P6" t="s">
         <v>22</v>
@@ -916,16 +960,28 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>124</v>
+        <v>50</v>
+      </c>
+      <c r="C7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E7" t="s">
+        <v>53</v>
+      </c>
+      <c r="M7" t="s">
+        <v>54</v>
       </c>
       <c r="N7">
         <v>1</v>
       </c>
       <c r="O7" t="s">
-        <v>120</v>
+        <v>55</v>
       </c>
       <c r="P7" t="s">
         <v>22</v>
@@ -933,272 +989,310 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" t="s">
-        <v>38</v>
-      </c>
-      <c r="D8" t="s">
-        <v>39</v>
-      </c>
-      <c r="E8" t="s">
-        <v>40</v>
-      </c>
-      <c r="M8" t="s">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="N8">
         <v>1</v>
       </c>
       <c r="O8" t="s">
-        <v>42</v>
-      </c>
-      <c r="P8" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>8</v>
+      <c r="A9" t="s">
+        <v>125</v>
       </c>
       <c r="B9" t="s">
-        <v>97</v>
-      </c>
-      <c r="C9" t="s">
-        <v>92</v>
+        <v>126</v>
       </c>
       <c r="N9">
         <v>1</v>
       </c>
       <c r="O9" t="s">
-        <v>43</v>
-      </c>
-      <c r="P9" t="s">
-        <v>44</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>109</v>
+      <c r="B10" t="s">
+        <v>63</v>
       </c>
       <c r="C10" t="s">
-        <v>92</v>
+        <v>128</v>
       </c>
       <c r="N10">
         <v>1</v>
       </c>
       <c r="O10" t="s">
-        <v>110</v>
+        <v>64</v>
       </c>
       <c r="P10" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A11">
-        <v>10</v>
+      <c r="A11" t="s">
+        <v>84</v>
       </c>
       <c r="B11" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="C11" t="s">
-        <v>92</v>
+        <v>72</v>
+      </c>
+      <c r="D11" t="s">
+        <v>73</v>
+      </c>
+      <c r="E11" t="s">
+        <v>74</v>
+      </c>
+      <c r="F11" t="s">
+        <v>75</v>
+      </c>
+      <c r="G11" t="s">
+        <v>76</v>
       </c>
       <c r="N11">
         <v>1</v>
       </c>
       <c r="O11" t="s">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="P11" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="C12" t="s">
-        <v>92</v>
+        <v>102</v>
+      </c>
+      <c r="D12" t="s">
+        <v>103</v>
+      </c>
+      <c r="E12" t="s">
+        <v>104</v>
       </c>
       <c r="N12">
         <v>1</v>
       </c>
       <c r="O12" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="P12" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>12</v>
+      <c r="A13" t="s">
+        <v>87</v>
       </c>
       <c r="B13" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="C13" t="s">
-        <v>92</v>
+        <v>72</v>
+      </c>
+      <c r="D13" t="s">
+        <v>73</v>
+      </c>
+      <c r="E13" t="s">
+        <v>74</v>
+      </c>
+      <c r="F13" t="s">
+        <v>75</v>
+      </c>
+      <c r="G13" t="s">
+        <v>76</v>
       </c>
       <c r="N13">
         <v>1</v>
       </c>
       <c r="O13" t="s">
-        <v>45</v>
+        <v>89</v>
       </c>
       <c r="P13" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>99</v>
+        <v>16</v>
       </c>
       <c r="C14" t="s">
-        <v>92</v>
+        <v>17</v>
+      </c>
+      <c r="D14" t="s">
+        <v>18</v>
+      </c>
+      <c r="E14" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" t="s">
+        <v>20</v>
       </c>
       <c r="N14">
         <v>1</v>
       </c>
       <c r="O14" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="P14" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A15">
-        <v>14</v>
+      <c r="A15" t="s">
+        <v>93</v>
       </c>
       <c r="B15" t="s">
-        <v>47</v>
+        <v>94</v>
+      </c>
+      <c r="C15" t="s">
+        <v>72</v>
+      </c>
+      <c r="D15" t="s">
+        <v>73</v>
+      </c>
+      <c r="E15" t="s">
+        <v>74</v>
+      </c>
+      <c r="F15" t="s">
+        <v>75</v>
+      </c>
+      <c r="G15" t="s">
+        <v>76</v>
       </c>
       <c r="N15">
         <v>1</v>
       </c>
       <c r="O15" t="s">
-        <v>48</v>
+        <v>95</v>
       </c>
       <c r="P15" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="M16" t="s">
-        <v>50</v>
-      </c>
-      <c r="N16">
-        <v>1</v>
-      </c>
-      <c r="O16" t="s">
-        <v>51</v>
+      <c r="A16" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="L16" s="4"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1">
+        <v>1</v>
+      </c>
+      <c r="O16" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="P16" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>115</v>
+        <v>78</v>
       </c>
       <c r="B17" t="s">
+        <v>79</v>
+      </c>
+      <c r="C17" t="s">
+        <v>72</v>
+      </c>
+      <c r="D17" t="s">
+        <v>73</v>
+      </c>
+      <c r="E17" t="s">
+        <v>74</v>
+      </c>
+      <c r="F17" t="s">
+        <v>75</v>
+      </c>
+      <c r="G17" t="s">
+        <v>76</v>
+      </c>
+      <c r="N17">
+        <v>1</v>
+      </c>
+      <c r="O17" t="s">
+        <v>80</v>
+      </c>
+      <c r="P17" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>7</v>
+      </c>
+      <c r="B18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18" t="s">
+        <v>128</v>
+      </c>
+      <c r="N18">
+        <v>1</v>
+      </c>
+      <c r="O18" t="s">
+        <v>60</v>
+      </c>
+      <c r="P18" t="s">
         <v>58</v>
       </c>
-      <c r="C17" t="s">
-        <v>52</v>
-      </c>
-      <c r="D17" t="s">
-        <v>53</v>
-      </c>
-      <c r="E17" t="s">
-        <v>54</v>
-      </c>
-      <c r="F17" t="s">
-        <v>55</v>
-      </c>
-      <c r="G17" t="s">
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>6</v>
+      </c>
+      <c r="B19" t="s">
         <v>56</v>
       </c>
-      <c r="N17">
-        <v>1</v>
-      </c>
-      <c r="O17" t="s">
-        <v>59</v>
-      </c>
-      <c r="P17" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>116</v>
-      </c>
-      <c r="B18" t="s">
-        <v>60</v>
-      </c>
-      <c r="C18" t="s">
-        <v>52</v>
-      </c>
-      <c r="D18" t="s">
-        <v>53</v>
-      </c>
-      <c r="E18" t="s">
-        <v>54</v>
-      </c>
-      <c r="F18" t="s">
-        <v>55</v>
-      </c>
-      <c r="G18" t="s">
-        <v>56</v>
-      </c>
-      <c r="N18">
-        <v>1</v>
-      </c>
-      <c r="O18" t="s">
-        <v>61</v>
-      </c>
-      <c r="P18" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>117</v>
-      </c>
-      <c r="B19" t="s">
-        <v>94</v>
-      </c>
       <c r="C19" t="s">
-        <v>52</v>
-      </c>
-      <c r="D19" t="s">
-        <v>53</v>
-      </c>
-      <c r="E19" t="s">
-        <v>54</v>
-      </c>
-      <c r="F19" t="s">
-        <v>55</v>
-      </c>
-      <c r="G19" t="s">
-        <v>56</v>
+        <v>128</v>
       </c>
       <c r="N19">
         <v>1</v>
@@ -1207,36 +1301,36 @@
         <v>57</v>
       </c>
       <c r="P19" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>118</v>
+        <v>81</v>
       </c>
       <c r="B20" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="C20" t="s">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="D20" t="s">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="E20" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
       <c r="F20" t="s">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="G20" t="s">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="N20">
         <v>1</v>
       </c>
       <c r="O20" t="s">
-        <v>102</v>
+        <v>83</v>
       </c>
       <c r="P20" t="s">
         <v>22</v>
@@ -1244,118 +1338,109 @@
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>119</v>
+        <v>90</v>
       </c>
       <c r="B21" t="s">
-        <v>62</v>
+        <v>91</v>
       </c>
       <c r="C21" t="s">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="D21" t="s">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="E21" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
       <c r="F21" t="s">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="G21" t="s">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="N21">
         <v>1</v>
       </c>
       <c r="O21" t="s">
-        <v>63</v>
+        <v>92</v>
       </c>
       <c r="P21" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A22">
-        <v>16</v>
+      <c r="A22" t="s">
+        <v>96</v>
       </c>
       <c r="B22" t="s">
-        <v>93</v>
-      </c>
-      <c r="M22" t="s">
-        <v>64</v>
+        <v>97</v>
+      </c>
+      <c r="C22" t="s">
+        <v>72</v>
+      </c>
+      <c r="D22" t="s">
+        <v>73</v>
+      </c>
+      <c r="E22" t="s">
+        <v>74</v>
+      </c>
+      <c r="F22" t="s">
+        <v>75</v>
+      </c>
+      <c r="G22" t="s">
+        <v>76</v>
       </c>
       <c r="N22">
         <v>1</v>
       </c>
       <c r="O22" t="s">
-        <v>65</v>
+        <v>98</v>
+      </c>
+      <c r="P22" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A23">
-        <v>17</v>
-      </c>
-      <c r="B23" t="s">
-        <v>66</v>
-      </c>
-      <c r="C23" t="s">
+        <v>11</v>
+      </c>
+      <c r="B23" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D23" t="s">
+      <c r="M23" t="s">
         <v>68</v>
       </c>
-      <c r="E23" t="s">
+      <c r="N23">
+        <v>1</v>
+      </c>
+      <c r="O23" t="s">
         <v>69</v>
-      </c>
-      <c r="N23">
-        <v>1</v>
-      </c>
-      <c r="O23" t="s">
-        <v>70</v>
-      </c>
-      <c r="P23" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A24">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="B24" t="s">
-        <v>71</v>
+        <v>45</v>
       </c>
       <c r="C24" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="D24" t="s">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="E24" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="F24" t="s">
-        <v>75</v>
-      </c>
-      <c r="G24" t="s">
-        <v>76</v>
-      </c>
-      <c r="H24" t="s">
-        <v>77</v>
-      </c>
-      <c r="I24" t="s">
-        <v>78</v>
-      </c>
-      <c r="J24" t="s">
-        <v>79</v>
-      </c>
-      <c r="K24" t="s">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="N24">
         <v>1</v>
       </c>
       <c r="O24" t="s">
-        <v>81</v>
+        <v>49</v>
       </c>
       <c r="P24" t="s">
         <v>22</v>
@@ -1363,28 +1448,43 @@
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A25">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B25" t="s">
-        <v>82</v>
+        <v>106</v>
       </c>
       <c r="C25" t="s">
-        <v>69</v>
+        <v>107</v>
       </c>
       <c r="D25" t="s">
-        <v>83</v>
+        <v>108</v>
       </c>
       <c r="E25" t="s">
-        <v>84</v>
-      </c>
-      <c r="M25" t="s">
-        <v>85</v>
+        <v>109</v>
+      </c>
+      <c r="F25" t="s">
+        <v>110</v>
+      </c>
+      <c r="G25" t="s">
+        <v>111</v>
+      </c>
+      <c r="H25" t="s">
+        <v>112</v>
+      </c>
+      <c r="I25" t="s">
+        <v>113</v>
+      </c>
+      <c r="J25" t="s">
+        <v>114</v>
+      </c>
+      <c r="K25" t="s">
+        <v>115</v>
       </c>
       <c r="N25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O25" t="s">
-        <v>86</v>
+        <v>116</v>
       </c>
       <c r="P25" t="s">
         <v>22</v>
@@ -1392,99 +1492,58 @@
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A26">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="B26" t="s">
-        <v>87</v>
+        <v>61</v>
       </c>
       <c r="C26" t="s">
-        <v>88</v>
-      </c>
-      <c r="D26" t="s">
-        <v>83</v>
-      </c>
-      <c r="E26" t="s">
-        <v>84</v>
-      </c>
-      <c r="M26" t="s">
-        <v>85</v>
+        <v>128</v>
       </c>
       <c r="N26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O26" t="s">
-        <v>89</v>
+        <v>62</v>
       </c>
       <c r="P26" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>114</v>
+      <c r="A27">
+        <v>2</v>
       </c>
       <c r="B27" t="s">
-        <v>122</v>
+        <v>23</v>
+      </c>
+      <c r="C27" t="s">
+        <v>24</v>
+      </c>
+      <c r="D27" t="s">
+        <v>25</v>
+      </c>
+      <c r="M27" t="s">
+        <v>26</v>
       </c>
       <c r="N27">
         <v>1</v>
       </c>
       <c r="O27" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>121</v>
-      </c>
-      <c r="B28" t="s">
-        <v>123</v>
-      </c>
-      <c r="N28">
-        <v>1</v>
-      </c>
-      <c r="O28" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
-        <v>111</v>
-      </c>
-      <c r="B29" t="s">
-        <v>90</v>
-      </c>
-      <c r="N29">
-        <v>1</v>
-      </c>
-      <c r="O29" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A33" s="1"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
-      <c r="F33" s="3"/>
-      <c r="G33" s="3"/>
-      <c r="H33" s="3"/>
-      <c r="I33" s="3"/>
-      <c r="J33" s="3"/>
-      <c r="K33" s="3"/>
-      <c r="L33" s="4"/>
-      <c r="M33" s="1"/>
-      <c r="N33" s="1"/>
-      <c r="O33" s="3"/>
+        <v>27</v>
+      </c>
+      <c r="P27" t="s">
+        <v>28</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P33" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P33">
-      <sortCondition ref="A1:A33"/>
+  <autoFilter ref="A1:P27" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P27">
+      <sortCondition ref="O1:O27"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>